<commit_message>
ajuste no diretorio de compras - MG
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56AD67B1-BC29-405E-BD1D-273CBE2A2E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8547E7-CA13-4788-B403-756929E90E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="73">
   <si>
     <t>Nome</t>
   </si>
@@ -253,6 +253,12 @@
   </si>
   <si>
     <t>KAROL_RODRIGUES</t>
+  </si>
+  <si>
+    <t>JOSUE_GOMES</t>
+  </si>
+  <si>
+    <t>BRUNO_BARBOSA</t>
   </si>
 </sst>
 </file>
@@ -345,7 +351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -360,6 +366,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -664,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -709,10 +718,10 @@
         <v>32</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="D3" s="4">
-        <v>5000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -737,10 +746,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="D5" s="4">
-        <v>8000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -880,7 +889,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -922,7 +931,7 @@
         <v>5</v>
       </c>
       <c r="D18" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1104,7 +1113,7 @@
         <v>5</v>
       </c>
       <c r="D31" s="4">
-        <v>3500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1245,6 +1254,34 @@
       </c>
       <c r="D41" s="4">
         <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D42" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D43" s="4">
+        <v>3500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige blacklist de vendedores ignorando nomes com espaço
Pedidos com comissão fixa exigem validação do comprador
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8547E7-CA13-4788-B403-756929E90E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92B95CA-0B54-4535-8DB7-2439D07F74E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="COORDENADORES" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">BLACKLIST_VENDEDORES!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">VENDEDORES!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="78">
   <si>
     <t>Nome</t>
   </si>
@@ -258,14 +259,29 @@
     <t>JOSUE_GOMES</t>
   </si>
   <si>
-    <t>BRUNO_BARBOSA</t>
+    <t>Bruno_Barbosa</t>
+  </si>
+  <si>
+    <t>RAFAEL_CAMARGOS</t>
+  </si>
+  <si>
+    <t>Nathan Lucca - Dev</t>
+  </si>
+  <si>
+    <t>SHIRLEY_RIBEIRO</t>
+  </si>
+  <si>
+    <t>PAULO_SOCORRO</t>
+  </si>
+  <si>
+    <t>JOAO_PEDRO_VITAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,6 +309,14 @@
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -351,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -371,6 +395,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -673,7 +698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -739,14 +764,14 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
+      <c r="A5" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="D5" s="4">
         <v>3500</v>
@@ -759,8 +784,8 @@
       <c r="B6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>52</v>
+      <c r="C6" s="5" t="s">
+        <v>5</v>
       </c>
       <c r="D6" s="4">
         <v>3500</v>
@@ -768,35 +793,35 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="4">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D8" s="4">
-        <v>12000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>4</v>
@@ -805,32 +830,32 @@
         <v>52</v>
       </c>
       <c r="D9" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D10" s="4">
-        <v>3500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D11" s="4">
         <v>0</v>
@@ -838,7 +863,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>4</v>
@@ -852,7 +877,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>4</v>
@@ -861,26 +886,26 @@
         <v>5</v>
       </c>
       <c r="D13" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="4">
-        <v>0</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>4</v>
@@ -894,24 +919,24 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4">
-        <v>20000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>5</v>
@@ -922,7 +947,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>4</v>
@@ -931,12 +956,12 @@
         <v>5</v>
       </c>
       <c r="D18" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>4</v>
@@ -950,69 +975,69 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D20" s="4">
-        <v>3500</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>63</v>
+      <c r="A21" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D22" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="4">
         <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="4">
-        <v>3500</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="D24" s="4">
         <v>3500</v>
@@ -1020,7 +1045,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>4</v>
@@ -1034,7 +1059,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>4</v>
@@ -1048,7 +1073,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>4</v>
@@ -1062,71 +1087,71 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D28" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>29</v>
+      <c r="A29" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D29" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D30" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="4">
-        <v>4000</v>
+      <c r="A31" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="5">
+        <v>3500</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="4">
+      <c r="A32" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="2">
         <v>3500</v>
       </c>
     </row>
@@ -1160,13 +1185,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D35" s="4">
         <v>3500</v>
@@ -1174,10 +1199,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>5</v>
@@ -1188,21 +1213,21 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="D37" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>4</v>
@@ -1216,76 +1241,122 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="B42" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D39" s="4">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C40" s="4" t="s">
+      <c r="D42" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D43" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D44" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D40" s="4">
+      <c r="D46" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D41" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D42" s="4">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D43" s="4">
-        <v>3500</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D45">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1294,7 +1365,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1312,71 +1383,90 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>22</v>
-      </c>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E18" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A15">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>